<commit_message>
feat: add data logging to Excel from buffer on program exit
</commit_message>
<xml_diff>
--- a/logs_detection_ur3.xlsx
+++ b/logs_detection_ur3.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="datalogs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +51,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,59 +424,922 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="29" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_detection</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>id_camera</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ai_model</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>detection_start_time</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>detection_end_time</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>duration_s</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>average_fps</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>average_model_accuracy</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>average_fps</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>min_distance_to_robot_mm</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>actual_robot_speed_scale</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>camera_id</t>
-        </is>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>average_inference_time_ms</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>tcp_x</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>tcp_y</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>tcp_z</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:32</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:37</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>125.3</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:38</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:38</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:39</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:42</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:45</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:48</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:48</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:48</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>114.9</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:49</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:49</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>105.3</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:50</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:55</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:56</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:56</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:56</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:56</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:58</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:59</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:06:59</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:03</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:04</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:04</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:04</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:06</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:06</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:07</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:08</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:08</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:08</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:10</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:11</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 19:07:11</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final ver. of .xlsx logger + added function flag to change modes (with/without robot) if wanna make only some test in program
</commit_message>
<xml_diff>
--- a/logs_detection_ur3.xlsx
+++ b/logs_detection_ur3.xlsx
@@ -424,22 +424,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="29" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,45 +466,50 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>hardware_setup</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>detection_start_time</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>detection_end_time</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>duration_s</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>average_fps</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>average_model_accuracy</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>average_inference_time_ms</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>tcp_x</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>tcp_y</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>tcp_z</t>
         </is>
@@ -518,7 +524,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>detection</t>
+          <t>requires checking</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -528,34 +534,39 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:32</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:37</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>5.7</v>
+          <t>2026-06-12 20:21:26</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:21:26</t>
+        </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>9</v>
+        <v>0.25</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0.84</v>
+        <v>11.1</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>125.3</v>
+        <v>0.33</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>0</v>
+        <v>296.9571666819675</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>-253.8521207407773</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>159.9343225224462</v>
       </c>
     </row>
     <row r="3">
@@ -567,7 +578,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>requires checking</t>
+          <t>detection</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -577,34 +588,39 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:38</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:38</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0.09</v>
+          <t>2026-06-12 20:21:27</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:21:33</t>
+        </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>13.6</v>
+        <v>5.93</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.29</v>
+        <v>11.6</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>63.5</v>
+        <v>0.84</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>76.7</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>0</v>
+        <v>99.90756300659746</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>0</v>
+        <v>-353.828669227107</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>159.188441579429</v>
       </c>
     </row>
     <row r="4">
@@ -616,7 +632,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>detection</t>
+          <t>requires checking</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -626,34 +642,39 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:39</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:42</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>3.06</v>
+          <t>2026-06-12 20:21:35</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:21:35</t>
+        </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>10.5</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.78</v>
+        <v>13.4</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>85.09999999999999</v>
+        <v>0.52</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>0</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0</v>
+        <v>341.3397527273858</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0</v>
+        <v>280.2562717224453</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>157.795804477444</v>
       </c>
     </row>
     <row r="5">
@@ -675,34 +696,39 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:45</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:48</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>3.08</v>
+          <t>2026-06-12 20:21:36</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:21:38</t>
+        </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>11.4</v>
+        <v>2.52</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.83</v>
+        <v>13.5</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>79.8</v>
+        <v>0.86</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>0</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>376.7113595730216</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0</v>
+        <v>219.7623234980509</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>158.3087053211889</v>
       </c>
     </row>
     <row r="6">
@@ -714,7 +740,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>requires checking</t>
+          <t>detection</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -724,34 +750,39 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:48</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:48</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0.1</v>
+          <t>2026-06-12 20:21:41</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:21:44</t>
+        </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>9.6</v>
+        <v>3.03</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0.27</v>
+        <v>12.3</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>114.9</v>
+        <v>0.83</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0</v>
+        <v>-76.20152753324054</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0</v>
+        <v>-339.2996084881519</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>157.7763816271687</v>
       </c>
     </row>
     <row r="7">
@@ -763,7 +794,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>requires checking</t>
+          <t>detection</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -773,34 +804,39 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:49</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:49</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0.1</v>
+          <t>2026-06-12 20:21:46</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:21:49</t>
+        </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>11.6</v>
+        <v>2.55</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0.26</v>
+        <v>12.6</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>105.3</v>
+        <v>0.79</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>0</v>
+        <v>301.2788443372388</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>329.5740642279305</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>157.2795201292647</v>
       </c>
     </row>
     <row r="8">
@@ -812,7 +848,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>detection</t>
+          <t>requires checking</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -822,34 +858,39 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:50</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:55</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>5.66</v>
+          <t>2026-06-12 20:21:52</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:21:52</t>
+        </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>11.6</v>
+        <v>0.15</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0.83</v>
+        <v>11.7</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>77.2</v>
+        <v>0.54</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
+        <v>71.8</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0</v>
+        <v>243.1125351940047</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0</v>
+        <v>-296.9921770766152</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>159.8146281694566</v>
       </c>
     </row>
     <row r="9">
@@ -861,7 +902,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>requires checking</t>
+          <t>detection</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -871,34 +912,39 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:56</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:56</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>0.07000000000000001</v>
+          <t>2026-06-12 20:21:52</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:21:56</t>
+        </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>12.8</v>
+        <v>4.42</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.28</v>
+        <v>11.6</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>64.59999999999999</v>
+        <v>0.73</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>0</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>0</v>
+        <v>-73.87175280977351</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>-340.1063557425869</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>157.8014161737684</v>
       </c>
     </row>
     <row r="10">
@@ -910,7 +956,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>requires checking</t>
+          <t>detection</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -920,34 +966,39 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:56</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:56</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>0.09</v>
+          <t>2026-06-12 20:22:00</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:03</t>
+        </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>13.6</v>
+        <v>3.23</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.29</v>
+        <v>12.1</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>80.40000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0</v>
+        <v>418.8146963824411</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0</v>
+        <v>35.5154103342377</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>159.3782133447754</v>
       </c>
     </row>
     <row r="11">
@@ -969,34 +1020,39 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:58</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:59</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>0.09</v>
+          <t>2026-06-12 20:22:05</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:06</t>
+        </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>10.6</v>
+        <v>0.08</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.32</v>
+        <v>13.6</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>66.40000000000001</v>
+        <v>0.49</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0</v>
+        <v>-53.4076737511806</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0</v>
+        <v>-346.4084668884195</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>158.0123231021371</v>
       </c>
     </row>
     <row r="12">
@@ -1018,34 +1074,39 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:06:59</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:03</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>4.01</v>
+          <t>2026-06-12 20:22:06</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:09</t>
+        </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>11.8</v>
+        <v>3.21</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.85</v>
+        <v>12.5</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>75.3</v>
+        <v>0.79</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>0</v>
+        <v>52.85119174163302</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>-358.65656689093</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>158.8907290696348</v>
       </c>
     </row>
     <row r="13">
@@ -1057,7 +1118,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>requires checking</t>
+          <t>detection</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1067,34 +1128,39 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:04</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:04</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>0.08</v>
+          <t>2026-06-12 20:22:12</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:15</t>
+        </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>12.9</v>
+        <v>3.13</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.28</v>
+        <v>12.2</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>69.59999999999999</v>
+        <v>0.75</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>0</v>
+        <v>367.140193872142</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>238.4883060488579</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>158.1612961552632</v>
       </c>
     </row>
     <row r="14">
@@ -1106,7 +1172,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>detection</t>
+          <t>requires checking</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1116,34 +1182,39 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:04</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:06</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>1.78</v>
+          <t>2026-06-12 20:22:15</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:15</t>
+        </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>11.6</v>
+        <v>0.08</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.77</v>
+        <v>12</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>78.59999999999999</v>
+        <v>0.31</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0</v>
+        <v>76.5</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>0</v>
+        <v>415.1425336790175</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>91.44757487264189</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>159.1150437150943</v>
       </c>
     </row>
     <row r="15">
@@ -1165,34 +1236,39 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:06</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:07</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>1.03</v>
+          <t>2026-06-12 20:22:17</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:19</t>
+        </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>12</v>
+        <v>1.33</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.6</v>
+        <v>12.1</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>74.90000000000001</v>
+        <v>0.74</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>0</v>
+        <v>73.7</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>0</v>
+        <v>-103.6589047793671</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>-328.3314874315122</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>157.4625163612595</v>
       </c>
     </row>
     <row r="16">
@@ -1214,34 +1290,39 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:08</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:08</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>0.16</v>
+          <t>2026-06-12 20:22:20</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:20</t>
+        </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>12.1</v>
+        <v>0.08</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.54</v>
+        <v>11.8</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>78.59999999999999</v>
+        <v>0.36</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>78.8</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>0</v>
+        <v>-52.15671284567581</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>-346.7492191563477</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>158.0247869494208</v>
       </c>
     </row>
     <row r="17">
@@ -1253,7 +1334,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>detection</t>
+          <t>requires checking</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1263,34 +1344,39 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:08</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:10</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>1.93</v>
+          <t>2026-06-12 20:22:20</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:20</t>
+        </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>12.2</v>
+        <v>0.08</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.61</v>
+        <v>13.2</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>72.09999999999999</v>
+        <v>0.35</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0</v>
+        <v>79.8</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>0</v>
+        <v>-24.29955387147018</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0</v>
+        <v>-353.0668205535091</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>158.2862028460158</v>
       </c>
     </row>
     <row r="18">
@@ -1312,33 +1398,902 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:11</t>
+          <t>cobot</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 19:07:11</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n">
+          <t>2026-06-12 20:22:21</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:21</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>80.09999999999999</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>171.3862910400345</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>-334.126006273644</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>159.5526008850337</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:22</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:22</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>406.2406675615518</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>-64.94020593570571</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>159.7359999180601</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:23</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:23</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>370.2841535153469</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>232.5809261024094</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>158.2086981205857</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:23</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:24</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>317.650514315408</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>311.1502494377624</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>157.4852516794919</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:24</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:31</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>29.72767461276764</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>-358.7550607309078</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>158.7261036950252</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:32</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:32</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>-52.15166846454035</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>-346.7505655854082</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>158.0248163273716</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:32</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:33</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>-118.056631387245</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>-321.4339714458717</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>157.2830277894036</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:33</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:33</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>-111.421285924351</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>-324.7161399390915</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>157.3670161978898</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:33</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:33</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
         <v>0.08</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="I26" s="2" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>-103.6236673275074</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>-328.3473744063875</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>157.4628458994333</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:33</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:34</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>-93.41583032696508</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>-332.746349598383</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>157.5837175694251</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:34</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:22:34</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>-78.3093921079562</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>-338.5535488268747</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>157.7534108541523</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:27:04</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:27:07</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>400.6011790672853</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>158.4479329304321</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>158.7336572215669</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>cobot</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:27:09</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:27:12</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="I30" s="2" t="n">
         <v>12.4</v>
       </c>
-      <c r="I18" s="2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="2" t="n">
+      <c r="J30" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>-117.7105141289481</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>-321.6096498958875</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>157.2874379390676</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:31:12</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:31:12</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:31:12</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:31:13</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:31:14</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:31:14</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:31:14</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:31:15</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>